<commit_message>
vaje za ipit latex, html
</commit_message>
<xml_diff>
--- a/10-razpredelnice/tockovanje.xlsx
+++ b/10-razpredelnice/tockovanje.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katja/Versioned/Predmeti/racunalniski-praktikum/vaje/03-excel/vaje2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zalakmetic/Documents/fmf/1. letnik/1. semester/računalniški praktikum/racunalniski-praktikum/10-razpredelnice/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4BC39C-E016-7A44-8583-BE6404D1B41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531DD9A3-0758-ED40-8009-B5F6336F1AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3180" yWindow="-26460" windowWidth="34160" windowHeight="23680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Točkovanje" sheetId="1" r:id="rId1"/>
@@ -1167,46 +1167,46 @@
     <row r="2" spans="2:23" ht="46" x14ac:dyDescent="0.2">
       <c r="D2" s="1"/>
       <c r="E2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="K2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="N2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="P2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="2:23" ht="45" x14ac:dyDescent="0.2">
@@ -1217,46 +1217,46 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="K3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="N3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="P3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R3" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" spans="2:23" ht="26" x14ac:dyDescent="0.3">
@@ -1281,32 +1281,32 @@
       <c r="D5" s="1">
         <v>2</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="G5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I5" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="J5" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="K5" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="L5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="M5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" s="8" t="s">
         <v>69</v>
@@ -1331,28 +1331,28 @@
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="Q6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R6" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1366,16 +1366,22 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>1</v>
+      <c r="E7" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N7" s="2" t="s">
@@ -1384,13 +1390,7 @@
       <c r="O7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P7" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="Q7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R7" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1404,25 +1404,25 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="N8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="Q8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R8" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1436,37 +1436,37 @@
       <c r="D9" s="1">
         <v>1</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>0</v>
+      <c r="E9" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="I9" s="2" t="s">
         <v>0</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="K9" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="L9" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="M9" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="N9" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R9" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1480,34 +1480,34 @@
       <c r="D10" s="1">
         <v>1</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>0</v>
+      <c r="E10" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>0</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="M10" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="N10" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R10" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1521,28 +1521,28 @@
       <c r="D11" s="1">
         <v>3</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="E11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>1</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="K11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="N11" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="P11" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="Q11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R11" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1556,31 +1556,31 @@
       <c r="D12" s="1">
         <v>2</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>0</v>
+      <c r="E12" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="L12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="s">
         <v>1</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R12" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1594,10 +1594,16 @@
       <c r="D13" s="1">
         <v>2</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="E13" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>1</v>
       </c>
       <c r="L13" s="2" t="s">
@@ -1606,16 +1612,10 @@
       <c r="N13" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O13" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="P13" s="2" t="s">
         <v>1</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R13" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1666,7 +1666,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>0</v>
@@ -1675,12 +1678,9 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O16" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P16" s="2" t="s">
@@ -1704,34 +1704,34 @@
         <v>2</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K17" s="2" t="s">
         <v>0</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="O17" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>0</v>
@@ -1768,8 +1768,11 @@
       <c r="J18" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="K18" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="L18" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>0</v>
@@ -1781,12 +1784,9 @@
         <v>0</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R18" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1822,7 +1822,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>0</v>
@@ -1834,7 +1834,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>0</v>
@@ -1863,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>0</v>
@@ -1874,9 +1874,6 @@
       <c r="K20" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L20" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="M20" s="2" t="s">
         <v>0</v>
       </c>
@@ -1884,6 +1881,9 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P20" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="s">
@@ -1919,7 +1919,13 @@
         <v>0</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>0</v>
@@ -1928,15 +1934,9 @@
         <v>0</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P21" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R21" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1959,7 +1959,10 @@
       <c r="G22" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -1969,9 +1972,6 @@
         <v>0</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O22" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P22" s="2" t="s">
@@ -1994,20 +1994,23 @@
       <c r="D23" s="1">
         <v>2</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>0</v>
+      <c r="E23" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="J23" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="K23" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>0</v>
@@ -2016,9 +2019,6 @@
         <v>0</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="O23" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P23" s="2" t="s">
@@ -2028,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="2:18" x14ac:dyDescent="0.2">
@@ -2128,19 +2128,19 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>0</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>0</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>0</v>
@@ -2152,7 +2152,7 @@
         <v>0</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q27" s="2" t="s">
         <v>0</v>
@@ -2187,7 +2187,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>0</v>
@@ -2202,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>0</v>
@@ -2240,11 +2240,14 @@
         <v>0</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="L29" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="M29" s="2" t="s">
         <v>0</v>
       </c>
@@ -2252,10 +2255,7 @@
         <v>0</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P29" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q29" s="2" t="s">
         <v>0</v>
@@ -2275,10 +2275,10 @@
         <v>1</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>0</v>
@@ -2286,6 +2286,9 @@
       <c r="I30" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="J30" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K30" s="2" t="s">
         <v>0</v>
       </c>
@@ -2296,9 +2299,6 @@
         <v>0</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O30" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P30" s="2" t="s">
@@ -2321,16 +2321,16 @@
       <c r="D31" s="1">
         <v>1</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="E31" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="s">
         <v>0</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P31" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2344,9 +2344,6 @@
       <c r="D32" s="1">
         <v>1</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="F32" s="2" t="s">
         <v>0</v>
       </c>
@@ -2359,19 +2356,22 @@
       <c r="I32" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="J32" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K32" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L32" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="M32" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O32" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="2" t="s">
+      <c r="N32" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="R32" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2397,20 +2397,20 @@
       <c r="H33" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I33" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K33" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>0</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="s">
-        <v>1</v>
       </c>
       <c r="Q33" s="2" t="s">
         <v>0</v>
@@ -2439,11 +2439,14 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="J34" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K34" s="2" t="s">
         <v>0</v>
       </c>
@@ -2451,12 +2454,9 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O34" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P34" s="2" t="s">
@@ -2480,16 +2480,16 @@
         <v>1</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>0</v>
@@ -2500,23 +2500,23 @@
       <c r="K35" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="L35" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="M35" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P35" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="Q35" s="2" t="s">
         <v>1</v>
       </c>
       <c r="R35" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.2">
@@ -2541,19 +2541,19 @@
       <c r="H36" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I36" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K36" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="L36" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O36" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P36" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q36" s="2" t="s">
@@ -2573,22 +2573,22 @@
       <c r="D37" s="1">
         <v>1</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I37" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="K37" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="M37" s="2" t="s">
-        <v>0</v>
-      </c>
       <c r="N37" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O37" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q37" s="2" t="s">
@@ -2620,13 +2620,13 @@
       <c r="H38" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="I38" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="J38" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="M38" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N38" s="2" t="s">
@@ -2665,7 +2665,10 @@
         <v>0</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>0</v>
@@ -2674,12 +2677,9 @@
         <v>1</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O39" s="2" t="s">
         <v>0</v>
       </c>
       <c r="P39" s="2" t="s">
@@ -2706,7 +2706,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>0</v>
@@ -2723,23 +2723,23 @@
       <c r="K40" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="L40" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="M40" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="P40" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="Q40" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R40" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="2:18" x14ac:dyDescent="0.2">
@@ -2752,11 +2752,8 @@
       <c r="D41" s="1">
         <v>3</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>1</v>
+      <c r="E41" s="2" t="s">
+        <v>0</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>1</v>
@@ -2764,16 +2761,19 @@
       <c r="J41" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="K41" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="N41" s="2" t="s">
         <v>0</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="R41" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2791,27 +2791,27 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>1</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
         <v>1</v>
       </c>
       <c r="K42" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2" t="s">
         <v>1</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>1</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O42" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="P42" s="2" t="s">
         <v>1</v>
       </c>
       <c r="Q42" s="2" t="s">
@@ -2861,6 +2861,9 @@
       <c r="R45" s="5"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" columnSort="1" ref="E2:R42">
+    <sortCondition ref="E2:R2"/>
+  </sortState>
   <mergeCells count="1">
     <mergeCell ref="T4:W4"/>
   </mergeCells>

</xml_diff>